<commit_message>
añadido fotos para jugadores y mejorado la insercion de nuevos futbolistas
</commit_message>
<xml_diff>
--- a/data/watford_players_login_info.xlsx
+++ b/data/watford_players_login_info.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,7 +425,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C42"/>
+  <dimension ref="A1:D42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -444,175 +444,219 @@
           <t>activo</t>
         </is>
       </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>photo_url</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Daniel Bachmann</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>141468</v>
+          <t>Alfie Marriott</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>495339</t>
+        </is>
       </c>
       <c r="C2" t="n">
         <v>1</v>
       </c>
+      <c r="D2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Francisco Sierralta</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>362761</v>
+          <t>Amin Nabizada</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>516143</t>
+        </is>
       </c>
       <c r="C3" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Mattie Pollock</t>
-        </is>
-      </c>
-      <c r="B4" t="n">
-        <v>368493</v>
+          <t>Angelo Ogbonna</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>23547</t>
+        </is>
       </c>
       <c r="C4" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>James Morris</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>425565</v>
+          <t>Antonio Tikvic</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>494112</t>
+        </is>
       </c>
       <c r="C5" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Ryan Andrews</t>
-        </is>
-      </c>
-      <c r="B6" t="n">
-        <v>470676</v>
+          <t>Caleb Wiley</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>433594</t>
+        </is>
       </c>
       <c r="C6" t="n">
         <v>1</v>
       </c>
+      <c r="D6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Jeremy Ngakia</t>
-        </is>
-      </c>
-      <c r="B7" t="n">
-        <v>390700</v>
+          <t>Daniel Bachmann</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>141468</t>
+        </is>
       </c>
       <c r="C7" t="n">
         <v>1</v>
       </c>
+      <c r="D7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Moussa Sissoko</t>
-        </is>
-      </c>
-      <c r="B8" t="n">
-        <v>29595</v>
+          <t>Daniel Jebbison</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>415163</t>
+        </is>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Tom Dele-Bashiru</t>
-        </is>
-      </c>
-      <c r="B9" t="n">
-        <v>350062</v>
+          <t>Edo Kayembe</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>363718</t>
+        </is>
       </c>
       <c r="C9" t="n">
         <v>1</v>
       </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Edo Kayembe</t>
-        </is>
-      </c>
-      <c r="B10" t="n">
-        <v>363718</v>
+          <t>Egil Selvik</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>372297</t>
+        </is>
       </c>
       <c r="C10" t="n">
         <v>1</v>
       </c>
+      <c r="D10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Giorgi Chakvetadze</t>
-        </is>
-      </c>
-      <c r="B11" t="n">
-        <v>363139</v>
+          <t>Festy Ebosele</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>408984</t>
+        </is>
       </c>
       <c r="C11" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Vakoun Bayo</t>
-        </is>
-      </c>
-      <c r="B12" t="n">
-        <v>383814</v>
+          <t>Francisco Sierralta</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>362761</t>
+        </is>
       </c>
       <c r="C12" t="n">
         <v>0</v>
       </c>
+      <c r="D12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Mileta Rajovic</t>
-        </is>
-      </c>
-      <c r="B13" t="n">
-        <v>498185</v>
+          <t>Giorgi Chakvetadze</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>363139</t>
+        </is>
       </c>
       <c r="C13" t="n">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>data/player_photos/363139.jpg</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Yasser Larouci</t>
-        </is>
-      </c>
-      <c r="B14" t="n">
-        <v>386971</v>
-      </c>
+          <t>Hector Kyprianou</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr"/>
       <c r="C14" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -620,355 +664,435 @@
           <t>Imrân Louza</t>
         </is>
       </c>
-      <c r="B15" t="n">
-        <v>367217</v>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>367217</t>
+        </is>
       </c>
       <c r="C15" t="n">
         <v>1</v>
       </c>
+      <c r="D15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Kwadwo Baah</t>
-        </is>
-      </c>
-      <c r="B16" t="n">
-        <v>384353</v>
+          <t>Jai-Dea Moulton</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>555487</t>
+        </is>
       </c>
       <c r="C16" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Rocco Vata</t>
-        </is>
-      </c>
-      <c r="B17" t="n">
-        <v>454349</v>
+          <t>James Abankwah</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>446988</t>
+        </is>
       </c>
       <c r="C17" t="n">
         <v>1</v>
       </c>
+      <c r="D17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Ken Sema</t>
-        </is>
-      </c>
-      <c r="B18" t="n">
-        <v>145392</v>
+          <t>James Morris</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>425565</t>
+        </is>
       </c>
       <c r="C18" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Jonathan Bond</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>81979</v>
+          <t>Jeremy Ngakia</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>390700</t>
+        </is>
       </c>
       <c r="C19" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Tom Ince</t>
-        </is>
-      </c>
-      <c r="B20" t="n">
-        <v>90918</v>
+          <t>Jonathan Bond</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>81979</t>
+        </is>
       </c>
       <c r="C20" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Ryan Porteous</t>
-        </is>
-      </c>
-      <c r="B21" t="n">
-        <v>388017</v>
+          <t>Ken Sema</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>145392</t>
+        </is>
       </c>
       <c r="C21" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Mamadou Doumbia</t>
-        </is>
-      </c>
-      <c r="B22" t="n">
-        <v>512775</v>
+          <t>Kwadwo Baah</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>384353</t>
+        </is>
       </c>
       <c r="C22" t="n">
         <v>1</v>
       </c>
+      <c r="D22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Angelo Ogbonna</t>
-        </is>
-      </c>
-      <c r="B23" t="n">
-        <v>23547</v>
+          <t>Kévin Keben</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>444726</t>
+        </is>
       </c>
       <c r="C23" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Festy Ebosele</t>
-        </is>
-      </c>
-      <c r="B24" t="n">
-        <v>408984</v>
+          <t>Leo Ramirez-Espain</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>526551</t>
+        </is>
       </c>
       <c r="C24" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Daniel Jebbison</t>
-        </is>
-      </c>
-      <c r="B25" t="n">
-        <v>415163</v>
-      </c>
+          <t>Luca Kjerrumgaard</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr"/>
       <c r="C25" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>Antonio Tikvic</t>
-        </is>
-      </c>
-      <c r="B26" t="n">
-        <v>494112</v>
+          <t>Mamadou Doumbia</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>512775</t>
+        </is>
       </c>
       <c r="C26" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>Alfie Marriott</t>
-        </is>
-      </c>
-      <c r="B27" t="n">
-        <v>495339</v>
-      </c>
+          <t>Marc Bola</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr"/>
       <c r="C27" t="n">
         <v>1</v>
       </c>
+      <c r="D27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>Pierre Dwomoh</t>
-        </is>
-      </c>
-      <c r="B28" t="n">
-        <v>403894</v>
+          <t>Mattie Pollock</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>368493</t>
+        </is>
       </c>
       <c r="C28" t="n">
         <v>1</v>
       </c>
+      <c r="D28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>Leo Ramirez-Espain</t>
-        </is>
-      </c>
-      <c r="B29" t="n">
-        <v>526551</v>
+          <t>Michael Adu-Poku</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>470678</t>
+        </is>
       </c>
       <c r="C29" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>Kévin Keben</t>
-        </is>
-      </c>
-      <c r="B30" t="n">
-        <v>444726</v>
+          <t>Mileta Rajovic</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>498185</t>
+        </is>
       </c>
       <c r="C30" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>Myles Roberts</t>
-        </is>
-      </c>
-      <c r="B31" t="n">
-        <v>479285</v>
+          <t>Moussa Sissoko</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>29595</t>
+        </is>
       </c>
       <c r="C31" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>James Abankwah</t>
-        </is>
-      </c>
-      <c r="B32" t="n">
-        <v>446988</v>
+          <t>Myles Roberts</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>479285</t>
+        </is>
       </c>
       <c r="C32" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Amin Nabizada</t>
-        </is>
-      </c>
-      <c r="B33" t="n">
-        <v>516143</v>
+          <t>Pierre Dwomoh</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>403894</t>
+        </is>
       </c>
       <c r="C33" t="n">
         <v>1</v>
       </c>
+      <c r="D33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Egil Selvik</t>
-        </is>
-      </c>
-      <c r="B34" t="n">
-        <v>372297</v>
+          <t>Rocco Vata</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>454349</t>
+        </is>
       </c>
       <c r="C34" t="n">
         <v>1</v>
       </c>
+      <c r="D34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Michael Adu-Poku</t>
-        </is>
-      </c>
-      <c r="B35" t="n">
-        <v>470678</v>
+          <t>Ryan Andrews</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>470676</t>
+        </is>
       </c>
       <c r="C35" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Caleb Wiley</t>
-        </is>
-      </c>
-      <c r="B36" t="n">
-        <v>433594</v>
+          <t>Ryan Porteous</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>388017</t>
+        </is>
       </c>
       <c r="C36" t="n">
         <v>1</v>
       </c>
+      <c r="D36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Zavier Massiah-Edwards</t>
-        </is>
-      </c>
-      <c r="B37" t="n">
-        <v>521224</v>
+          <t>Tom Dele-Bashiru</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>350062</t>
+        </is>
       </c>
       <c r="C37" t="n">
         <v>1</v>
       </c>
+      <c r="D37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>Jai-Dea Moulton</t>
-        </is>
-      </c>
-      <c r="B38" t="n">
-        <v>555487</v>
+          <t>Tom Ince</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>90918</t>
+        </is>
       </c>
       <c r="C38" t="n">
-        <v>0</v>
-      </c>
+        <v>1</v>
+      </c>
+      <c r="D38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>Vivaldo Semedo</t>
-        </is>
-      </c>
-      <c r="B39" t="inlineStr"/>
+          <t>Vakoun Bayo</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>383814</t>
+        </is>
+      </c>
       <c r="C39" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Hector Kyprianou</t>
+          <t>Vivaldo Semedo</t>
         </is>
       </c>
       <c r="B40" t="inlineStr"/>
       <c r="C40" t="n">
         <v>1</v>
       </c>
+      <c r="D40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Marc Bola</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr"/>
+          <t>Yasser Larouci</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>386971</t>
+        </is>
+      </c>
       <c r="C41" t="n">
-        <v>1</v>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="D41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Luca Kjerrumgaard</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr"/>
+          <t>Zavier Massiah-Edwards</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>521224</t>
+        </is>
+      </c>
       <c r="C42" t="n">
         <v>1</v>
       </c>
+      <c r="D42" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
cambiado id interno, añadir nuevos jugadores, pdf reporte
</commit_message>
<xml_diff>
--- a/data/watford_players_login_info.xlsx
+++ b/data/watford_players_login_info.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -425,26 +425,36 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D42"/>
+  <dimension ref="A1:F42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
+          <t>internal_id</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
           <t>playerName</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>playerId</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>internal_position</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>activo</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>photo_url</t>
         </is>
@@ -453,194 +463,270 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
+          <t>INT-00001</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
           <t>Alfie Marriott</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr">
+      <c r="C2" t="inlineStr">
         <is>
           <t>495339</t>
         </is>
       </c>
-      <c r="C2" t="n">
-        <v>1</v>
-      </c>
       <c r="D2" t="inlineStr"/>
+      <c r="E2" t="n">
+        <v>1</v>
+      </c>
+      <c r="F2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>INT-00002</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
           <t>Amin Nabizada</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
+      <c r="C3" t="inlineStr">
         <is>
           <t>516143</t>
         </is>
       </c>
-      <c r="C3" t="n">
-        <v>1</v>
-      </c>
       <c r="D3" t="inlineStr"/>
+      <c r="E3" t="n">
+        <v>1</v>
+      </c>
+      <c r="F3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
+          <t>INT-00003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
           <t>Angelo Ogbonna</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
+      <c r="C4" t="inlineStr">
         <is>
           <t>23547</t>
         </is>
       </c>
-      <c r="C4" t="n">
+      <c r="D4" t="inlineStr"/>
+      <c r="E4" t="n">
         <v>0</v>
       </c>
-      <c r="D4" t="inlineStr"/>
+      <c r="F4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
+          <t>INT-00004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
           <t>Antonio Tikvic</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr">
+      <c r="C5" t="inlineStr">
         <is>
           <t>494112</t>
         </is>
       </c>
-      <c r="C5" t="n">
+      <c r="D5" t="inlineStr"/>
+      <c r="E5" t="n">
         <v>0</v>
       </c>
-      <c r="D5" t="inlineStr"/>
+      <c r="F5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
+          <t>INT-00005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
           <t>Caleb Wiley</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr">
+      <c r="C6" t="inlineStr">
         <is>
           <t>433594</t>
         </is>
       </c>
-      <c r="C6" t="n">
-        <v>1</v>
-      </c>
       <c r="D6" t="inlineStr"/>
+      <c r="E6" t="n">
+        <v>1</v>
+      </c>
+      <c r="F6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
+          <t>INT-00006</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
           <t>Daniel Bachmann</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr">
+      <c r="C7" t="inlineStr">
         <is>
           <t>141468</t>
         </is>
       </c>
-      <c r="C7" t="n">
-        <v>1</v>
-      </c>
       <c r="D7" t="inlineStr"/>
+      <c r="E7" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>data/player_photos/141468.jpg</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
+          <t>INT-00007</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>Daniel Jebbison</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr">
+      <c r="C8" t="inlineStr">
         <is>
           <t>415163</t>
         </is>
       </c>
-      <c r="C8" t="n">
+      <c r="D8" t="inlineStr"/>
+      <c r="E8" t="n">
         <v>0</v>
       </c>
-      <c r="D8" t="inlineStr"/>
+      <c r="F8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>INT-00008</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
           <t>Edo Kayembe</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr">
+      <c r="C9" t="inlineStr">
         <is>
           <t>363718</t>
         </is>
       </c>
-      <c r="C9" t="n">
-        <v>1</v>
-      </c>
       <c r="D9" t="inlineStr"/>
+      <c r="E9" t="n">
+        <v>1</v>
+      </c>
+      <c r="F9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>INT-00009</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
           <t>Egil Selvik</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>372297</t>
         </is>
       </c>
-      <c r="C10" t="n">
-        <v>1</v>
-      </c>
       <c r="D10" t="inlineStr"/>
+      <c r="E10" t="n">
+        <v>1</v>
+      </c>
+      <c r="F10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
+          <t>INT-00010</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
           <t>Festy Ebosele</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>408984</t>
         </is>
       </c>
-      <c r="C11" t="n">
+      <c r="D11" t="inlineStr"/>
+      <c r="E11" t="n">
         <v>0</v>
       </c>
-      <c r="D11" t="inlineStr"/>
+      <c r="F11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>INT-00011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
           <t>Francisco Sierralta</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr">
+      <c r="C12" t="inlineStr">
         <is>
           <t>362761</t>
         </is>
       </c>
-      <c r="C12" t="n">
+      <c r="D12" t="inlineStr"/>
+      <c r="E12" t="n">
         <v>0</v>
       </c>
-      <c r="D12" t="inlineStr"/>
+      <c r="F12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>INT-00012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>Giorgi Chakvetadze</t>
         </is>
       </c>
-      <c r="B13" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>363139</t>
         </is>
       </c>
-      <c r="C13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D13" t="inlineStr">
+      <c r="D13" t="inlineStr"/>
+      <c r="E13" t="n">
+        <v>1</v>
+      </c>
+      <c r="F13" t="inlineStr">
         <is>
           <t>data/player_photos/363139.jpg</t>
         </is>
@@ -649,450 +735,624 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
+          <t>INT-00013</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>Hector Kyprianou</t>
         </is>
       </c>
-      <c r="B14" t="inlineStr"/>
-      <c r="C14" t="n">
-        <v>1</v>
-      </c>
+      <c r="C14" t="inlineStr"/>
       <c r="D14" t="inlineStr"/>
+      <c r="E14" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>INT-00014</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
           <t>Imrân Louza</t>
         </is>
       </c>
-      <c r="B15" t="inlineStr">
+      <c r="C15" t="inlineStr">
         <is>
           <t>367217</t>
         </is>
       </c>
-      <c r="C15" t="n">
-        <v>1</v>
-      </c>
       <c r="D15" t="inlineStr"/>
+      <c r="E15" t="n">
+        <v>1</v>
+      </c>
+      <c r="F15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
+          <t>INT-00015</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
           <t>Jai-Dea Moulton</t>
         </is>
       </c>
-      <c r="B16" t="inlineStr">
+      <c r="C16" t="inlineStr">
         <is>
           <t>555487</t>
         </is>
       </c>
-      <c r="C16" t="n">
+      <c r="D16" t="inlineStr"/>
+      <c r="E16" t="n">
         <v>0</v>
       </c>
-      <c r="D16" t="inlineStr"/>
+      <c r="F16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
+          <t>INT-00016</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
           <t>James Abankwah</t>
         </is>
       </c>
-      <c r="B17" t="inlineStr">
+      <c r="C17" t="inlineStr">
         <is>
           <t>446988</t>
         </is>
       </c>
-      <c r="C17" t="n">
-        <v>1</v>
-      </c>
       <c r="D17" t="inlineStr"/>
+      <c r="E17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
+          <t>INT-00017</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
           <t>James Morris</t>
         </is>
       </c>
-      <c r="B18" t="inlineStr">
+      <c r="C18" t="inlineStr">
         <is>
           <t>425565</t>
         </is>
       </c>
-      <c r="C18" t="n">
-        <v>1</v>
-      </c>
       <c r="D18" t="inlineStr"/>
+      <c r="E18" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
+          <t>INT-00018</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
           <t>Jeremy Ngakia</t>
         </is>
       </c>
-      <c r="B19" t="inlineStr">
+      <c r="C19" t="inlineStr">
         <is>
           <t>390700</t>
         </is>
       </c>
-      <c r="C19" t="n">
-        <v>1</v>
-      </c>
       <c r="D19" t="inlineStr"/>
+      <c r="E19" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
+          <t>INT-00019</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
           <t>Jonathan Bond</t>
         </is>
       </c>
-      <c r="B20" t="inlineStr">
+      <c r="C20" t="inlineStr">
         <is>
           <t>81979</t>
         </is>
       </c>
-      <c r="C20" t="n">
-        <v>0</v>
-      </c>
       <c r="D20" t="inlineStr"/>
+      <c r="E20" t="n">
+        <v>1</v>
+      </c>
+      <c r="F20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>INT-00020</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
           <t>Ken Sema</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="C21" t="inlineStr">
         <is>
           <t>145392</t>
         </is>
       </c>
-      <c r="C21" t="n">
+      <c r="D21" t="inlineStr"/>
+      <c r="E21" t="n">
         <v>0</v>
       </c>
-      <c r="D21" t="inlineStr"/>
+      <c r="F21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
+          <t>INT-00021</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
           <t>Kwadwo Baah</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="C22" t="inlineStr">
         <is>
           <t>384353</t>
         </is>
       </c>
-      <c r="C22" t="n">
-        <v>1</v>
-      </c>
       <c r="D22" t="inlineStr"/>
+      <c r="E22" t="n">
+        <v>1</v>
+      </c>
+      <c r="F22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
+          <t>INT-00022</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
           <t>Kévin Keben</t>
         </is>
       </c>
-      <c r="B23" t="inlineStr">
+      <c r="C23" t="inlineStr">
         <is>
           <t>444726</t>
         </is>
       </c>
-      <c r="C23" t="n">
-        <v>1</v>
-      </c>
       <c r="D23" t="inlineStr"/>
+      <c r="E23" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>INT-00023</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
           <t>Leo Ramirez-Espain</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="C24" t="inlineStr">
         <is>
           <t>526551</t>
         </is>
       </c>
-      <c r="C24" t="n">
-        <v>1</v>
-      </c>
       <c r="D24" t="inlineStr"/>
+      <c r="E24" t="n">
+        <v>1</v>
+      </c>
+      <c r="F24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
+          <t>INT-00024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
           <t>Luca Kjerrumgaard</t>
         </is>
       </c>
-      <c r="B25" t="inlineStr"/>
-      <c r="C25" t="n">
-        <v>1</v>
-      </c>
+      <c r="C25" t="inlineStr"/>
       <c r="D25" t="inlineStr"/>
+      <c r="E25" t="n">
+        <v>1</v>
+      </c>
+      <c r="F25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
+          <t>INT-00025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
           <t>Mamadou Doumbia</t>
         </is>
       </c>
-      <c r="B26" t="inlineStr">
+      <c r="C26" t="inlineStr">
         <is>
           <t>512775</t>
         </is>
       </c>
-      <c r="C26" t="n">
-        <v>1</v>
-      </c>
       <c r="D26" t="inlineStr"/>
+      <c r="E26" t="n">
+        <v>1</v>
+      </c>
+      <c r="F26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
+          <t>INT-00026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
           <t>Marc Bola</t>
         </is>
       </c>
-      <c r="B27" t="inlineStr"/>
-      <c r="C27" t="n">
-        <v>1</v>
-      </c>
+      <c r="C27" t="inlineStr"/>
       <c r="D27" t="inlineStr"/>
+      <c r="E27" t="n">
+        <v>1</v>
+      </c>
+      <c r="F27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
+          <t>INT-00027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
           <t>Mattie Pollock</t>
         </is>
       </c>
-      <c r="B28" t="inlineStr">
+      <c r="C28" t="inlineStr">
         <is>
           <t>368493</t>
         </is>
       </c>
-      <c r="C28" t="n">
-        <v>1</v>
-      </c>
       <c r="D28" t="inlineStr"/>
+      <c r="E28" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
+          <t>INT-00028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
           <t>Michael Adu-Poku</t>
         </is>
       </c>
-      <c r="B29" t="inlineStr">
+      <c r="C29" t="inlineStr">
         <is>
           <t>470678</t>
         </is>
       </c>
-      <c r="C29" t="n">
+      <c r="D29" t="inlineStr"/>
+      <c r="E29" t="n">
         <v>0</v>
       </c>
-      <c r="D29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>INT-00029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
           <t>Mileta Rajovic</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="C30" t="inlineStr">
         <is>
           <t>498185</t>
         </is>
       </c>
-      <c r="C30" t="n">
+      <c r="D30" t="inlineStr"/>
+      <c r="E30" t="n">
         <v>0</v>
       </c>
-      <c r="D30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
+          <t>INT-00030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
           <t>Moussa Sissoko</t>
         </is>
       </c>
-      <c r="B31" t="inlineStr">
+      <c r="C31" t="inlineStr">
         <is>
           <t>29595</t>
         </is>
       </c>
-      <c r="C31" t="n">
-        <v>1</v>
-      </c>
       <c r="D31" t="inlineStr"/>
+      <c r="E31" t="n">
+        <v>1</v>
+      </c>
+      <c r="F31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
+          <t>INT-00031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
           <t>Myles Roberts</t>
         </is>
       </c>
-      <c r="B32" t="inlineStr">
+      <c r="C32" t="inlineStr">
         <is>
           <t>479285</t>
         </is>
       </c>
-      <c r="C32" t="n">
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" t="n">
         <v>0</v>
       </c>
-      <c r="D32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
+          <t>INT-00032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
           <t>Pierre Dwomoh</t>
         </is>
       </c>
-      <c r="B33" t="inlineStr">
+      <c r="C33" t="inlineStr">
         <is>
           <t>403894</t>
         </is>
       </c>
-      <c r="C33" t="n">
-        <v>1</v>
-      </c>
       <c r="D33" t="inlineStr"/>
+      <c r="E33" t="n">
+        <v>1</v>
+      </c>
+      <c r="F33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
+          <t>INT-00033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
           <t>Rocco Vata</t>
         </is>
       </c>
-      <c r="B34" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>454349</t>
         </is>
       </c>
-      <c r="C34" t="n">
-        <v>1</v>
-      </c>
       <c r="D34" t="inlineStr"/>
+      <c r="E34" t="n">
+        <v>1</v>
+      </c>
+      <c r="F34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
+          <t>INT-00034</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
           <t>Ryan Andrews</t>
         </is>
       </c>
-      <c r="B35" t="inlineStr">
+      <c r="C35" t="inlineStr">
         <is>
           <t>470676</t>
         </is>
       </c>
-      <c r="C35" t="n">
-        <v>1</v>
-      </c>
       <c r="D35" t="inlineStr"/>
+      <c r="E35" t="n">
+        <v>1</v>
+      </c>
+      <c r="F35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
+          <t>INT-00035</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
           <t>Ryan Porteous</t>
         </is>
       </c>
-      <c r="B36" t="inlineStr">
+      <c r="C36" t="inlineStr">
         <is>
           <t>388017</t>
         </is>
       </c>
-      <c r="C36" t="n">
-        <v>1</v>
-      </c>
       <c r="D36" t="inlineStr"/>
+      <c r="E36" t="n">
+        <v>1</v>
+      </c>
+      <c r="F36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
+          <t>INT-00036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
           <t>Tom Dele-Bashiru</t>
         </is>
       </c>
-      <c r="B37" t="inlineStr">
+      <c r="C37" t="inlineStr">
         <is>
           <t>350062</t>
         </is>
       </c>
-      <c r="C37" t="n">
-        <v>1</v>
-      </c>
       <c r="D37" t="inlineStr"/>
+      <c r="E37" t="n">
+        <v>1</v>
+      </c>
+      <c r="F37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
+          <t>INT-00037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
           <t>Tom Ince</t>
         </is>
       </c>
-      <c r="B38" t="inlineStr">
+      <c r="C38" t="inlineStr">
         <is>
           <t>90918</t>
         </is>
       </c>
-      <c r="C38" t="n">
-        <v>1</v>
-      </c>
       <c r="D38" t="inlineStr"/>
+      <c r="E38" t="n">
+        <v>1</v>
+      </c>
+      <c r="F38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
+          <t>INT-00038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
           <t>Vakoun Bayo</t>
         </is>
       </c>
-      <c r="B39" t="inlineStr">
+      <c r="C39" t="inlineStr">
         <is>
           <t>383814</t>
         </is>
       </c>
-      <c r="C39" t="n">
+      <c r="D39" t="inlineStr"/>
+      <c r="E39" t="n">
         <v>0</v>
       </c>
-      <c r="D39" t="inlineStr"/>
+      <c r="F39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
+          <t>INT-00039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
           <t>Vivaldo Semedo</t>
         </is>
       </c>
-      <c r="B40" t="inlineStr"/>
-      <c r="C40" t="n">
-        <v>1</v>
-      </c>
+      <c r="C40" t="inlineStr"/>
       <c r="D40" t="inlineStr"/>
+      <c r="E40" t="n">
+        <v>1</v>
+      </c>
+      <c r="F40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
+          <t>INT-00040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
           <t>Yasser Larouci</t>
         </is>
       </c>
-      <c r="B41" t="inlineStr">
+      <c r="C41" t="inlineStr">
         <is>
           <t>386971</t>
         </is>
       </c>
-      <c r="C41" t="n">
+      <c r="D41" t="inlineStr"/>
+      <c r="E41" t="n">
         <v>0</v>
       </c>
-      <c r="D41" t="inlineStr"/>
+      <c r="F41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
+          <t>INT-00041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
           <t>Zavier Massiah-Edwards</t>
         </is>
       </c>
-      <c r="B42" t="inlineStr">
+      <c r="C42" t="inlineStr">
         <is>
           <t>521224</t>
         </is>
       </c>
-      <c r="C42" t="n">
-        <v>1</v>
-      </c>
       <c r="D42" t="inlineStr"/>
+      <c r="E42" t="n">
+        <v>1</v>
+      </c>
+      <c r="F42" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>